<commit_message>
Update binary files for exporter and formato templates
</commit_message>
<xml_diff>
--- a/templates/formato100.xlsx
+++ b/templates/formato100.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e039d0c270e9facf/Desktop/Developer/UANL---LABORATORIO-DE-ALIMENTOS-MEDICAMENTOS-Y-TOXICOLOGIA/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0B372F3-DC7E-4CCB-A2F2-2322F9ACB1D9}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="8_{47FAC42F-AC07-43D6-8172-01CEADEBF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF4AD8F4-7B5A-47B0-BFC9-67872A767946}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1CB8A4CE-E91B-448F-9BE6-E546BA7C8907}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>1. TABLA DE INFORMACIÓN NUTRIMENTAL (DECLARACIÓN NUTRIMENTAL)</t>
   </si>
   <si>
-    <t>Por 100 mL</t>
-  </si>
-  <si>
     <t>Contenido energético</t>
   </si>
   <si>
@@ -93,6 +90,9 @@
   </si>
   <si>
     <t xml:space="preserve">MUESTRA: </t>
+  </si>
+  <si>
+    <t>Por 100 g</t>
   </si>
 </sst>
 </file>
@@ -354,9 +354,48 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -374,45 +413,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -556,10 +556,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -895,28 +891,28 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -944,7 +940,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B8" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
@@ -956,25 +952,25 @@
       <c r="J8" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
+      <c r="B12" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F13" s="13"/>
@@ -991,17 +987,17 @@
       <c r="J14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="B15" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="24"/>
+      <c r="B15" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="36"/>
+      <c r="J15" s="37"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
@@ -1010,7 +1006,7 @@
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="3"/>
       <c r="C17" s="17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D17" s="17"/>
       <c r="E17" s="10"/>
@@ -1023,7 +1019,7 @@
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
       <c r="C18" s="17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D18" s="17"/>
       <c r="E18" s="12"/>
@@ -1035,7 +1031,7 @@
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
       <c r="C19" s="18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D19" s="18"/>
       <c r="E19" s="18"/>
@@ -1050,22 +1046,22 @@
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="G20" s="21"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="33"/>
+      <c r="F20" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="34"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
       <c r="J20" s="8"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
-      <c r="C21" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="37"/>
+      <c r="C21" s="32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="20"/>
       <c r="G21" s="12"/>
       <c r="H21" s="10"/>
       <c r="I21" s="10"/>
@@ -1073,12 +1069,12 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
-      <c r="C22" s="35" t="s">
-        <v>3</v>
-      </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="38"/>
+      <c r="C22" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="21"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
@@ -1086,12 +1082,12 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="35" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="38"/>
+      <c r="C23" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="21"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
@@ -1099,33 +1095,33 @@
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="37"/>
+      <c r="C24" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="20"/>
       <c r="J24" s="8"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" s="3"/>
-      <c r="C25" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="37"/>
+      <c r="C25" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="20"/>
       <c r="G25" s="19"/>
       <c r="J25" s="8"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
-      <c r="C26" s="36" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="38"/>
+      <c r="C26" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="21"/>
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
       <c r="I26" s="10"/>
@@ -1133,30 +1129,30 @@
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
-      <c r="C27" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="34"/>
-      <c r="F27" s="37"/>
+      <c r="C27" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="30"/>
+      <c r="F27" s="20"/>
       <c r="J27" s="8"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B28" s="3"/>
       <c r="C28" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D28" s="13"/>
-      <c r="F28" s="37"/>
+      <c r="F28" s="20"/>
       <c r="J28" s="8"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
-      <c r="C29" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="35"/>
+      <c r="C29" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="31"/>
       <c r="E29" s="10"/>
-      <c r="F29" s="38"/>
+      <c r="F29" s="21"/>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
       <c r="I29" s="10"/>
@@ -1164,12 +1160,12 @@
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
-      <c r="C30" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="20"/>
+      <c r="C30" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="32"/>
       <c r="E30" s="10"/>
-      <c r="F30" s="39"/>
+      <c r="F30" s="22"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
@@ -1187,56 +1183,60 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32" spans="2:10" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="31"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="31"/>
-      <c r="J32" s="32"/>
+      <c r="B32" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="28"/>
     </row>
     <row r="36" spans="2:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
+      <c r="B37" s="39"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
+      <c r="J37" s="39"/>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-      <c r="J38" s="27"/>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="23"/>
     </row>
     <row r="39" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="27"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="23"/>
     </row>
     <row r="44" spans="2:10" ht="58.15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="2:10" ht="59.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B37:J37"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="B39:J39"/>
     <mergeCell ref="A4:J4"/>
@@ -1253,10 +1253,6 @@
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B15:J15"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B37:J37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>